<commit_message>
Updated readme, cleaned file structure.
</commit_message>
<xml_diff>
--- a/SSEA_student_teams.xlsx
+++ b/SSEA_student_teams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\m.von-arnim\Documents\gitlab\m-vonarnim\ssea\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\m.von-arnim\Documents\gitlab\ssea_student_teams_repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10F12AE-F95F-4F35-8784-C5874CDA5772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97B543B-F255-4F68-A88E-2FC6FF2A5BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{7ED79F6E-3E07-4FE4-A152-12F8912DB878}"/>
+    <workbookView xWindow="-23148" yWindow="3036" windowWidth="23256" windowHeight="12576" xr2:uid="{7ED79F6E-3E07-4FE4-A152-12F8912DB878}"/>
   </bookViews>
   <sheets>
     <sheet name="SSEA_student_teams" sheetId="1" r:id="rId1"/>
@@ -3745,57 +3745,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F9AC9A0-6333-4726-AE68-2B1D81328658}">
   <dimension ref="A1:EI239"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" style="22" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" customWidth="1"/>
-    <col min="6" max="6" width="8.5546875" style="20" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="22" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="20" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="13" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="16.88671875" style="20" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="16.85546875" style="20" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5546875" customWidth="1"/>
-    <col min="13" max="13" width="7.5546875" style="22" customWidth="1"/>
-    <col min="14" max="14" width="6.44140625" style="22" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" style="22" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" customWidth="1"/>
+    <col min="13" max="13" width="7.5703125" style="22" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" style="22" customWidth="1"/>
+    <col min="15" max="15" width="8.85546875" style="22" customWidth="1"/>
     <col min="16" max="16" width="9" style="22" customWidth="1"/>
-    <col min="17" max="17" width="7.6640625" style="22" customWidth="1"/>
-    <col min="18" max="18" width="16.44140625" style="4" customWidth="1"/>
-    <col min="19" max="25" width="5.44140625" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="5.44140625" style="4" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="5.33203125" style="7" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="5.33203125" style="20" hidden="1" customWidth="1"/>
-    <col min="29" max="44" width="5.33203125" hidden="1" customWidth="1"/>
-    <col min="45" max="45" width="5.33203125" style="4" hidden="1" customWidth="1"/>
-    <col min="46" max="46" width="5.33203125" style="7" hidden="1" customWidth="1"/>
-    <col min="47" max="47" width="5.33203125" style="20" hidden="1" customWidth="1"/>
-    <col min="48" max="49" width="5.33203125" style="7" hidden="1" customWidth="1"/>
-    <col min="50" max="50" width="5.33203125" style="4" hidden="1" customWidth="1"/>
-    <col min="51" max="55" width="5.44140625" customWidth="1"/>
-    <col min="56" max="56" width="5.44140625" style="4" customWidth="1"/>
-    <col min="57" max="57" width="5.33203125" style="7" customWidth="1"/>
-    <col min="58" max="62" width="5.44140625" customWidth="1"/>
-    <col min="63" max="63" width="5.44140625" style="7" customWidth="1"/>
-    <col min="64" max="64" width="5.33203125" style="20" customWidth="1"/>
-    <col min="65" max="79" width="5.33203125" customWidth="1"/>
-    <col min="80" max="80" width="5.33203125" style="4" customWidth="1"/>
-    <col min="81" max="81" width="5.33203125" style="7" customWidth="1"/>
-    <col min="82" max="82" width="5.6640625" style="20" customWidth="1"/>
-    <col min="83" max="97" width="5.6640625" customWidth="1"/>
-    <col min="98" max="98" width="5.6640625" style="4" customWidth="1"/>
-    <col min="99" max="104" width="5.6640625" customWidth="1"/>
-    <col min="105" max="105" width="5.6640625" style="4" customWidth="1"/>
-    <col min="106" max="118" width="5.6640625" style="7" customWidth="1"/>
-    <col min="119" max="119" width="21.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="20.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="20.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="124" max="139" width="5.6640625" customWidth="1"/>
+    <col min="17" max="17" width="7.7109375" style="22" customWidth="1"/>
+    <col min="18" max="18" width="16.42578125" style="4" customWidth="1"/>
+    <col min="19" max="25" width="5.42578125" customWidth="1"/>
+    <col min="26" max="26" width="5.42578125" style="4" customWidth="1"/>
+    <col min="27" max="27" width="5.28515625" style="7" customWidth="1"/>
+    <col min="28" max="28" width="5.28515625" style="20" customWidth="1"/>
+    <col min="29" max="44" width="5.28515625" customWidth="1"/>
+    <col min="45" max="45" width="5.28515625" style="4" customWidth="1"/>
+    <col min="46" max="46" width="5.28515625" style="7" customWidth="1"/>
+    <col min="47" max="47" width="5.28515625" style="20" customWidth="1"/>
+    <col min="48" max="49" width="5.28515625" style="7" customWidth="1"/>
+    <col min="50" max="50" width="5.28515625" style="4" customWidth="1"/>
+    <col min="51" max="55" width="5.42578125" customWidth="1"/>
+    <col min="56" max="56" width="5.42578125" style="4" customWidth="1"/>
+    <col min="57" max="57" width="5.28515625" style="7" customWidth="1"/>
+    <col min="58" max="62" width="5.42578125" customWidth="1"/>
+    <col min="63" max="63" width="5.42578125" style="7" customWidth="1"/>
+    <col min="64" max="64" width="5.28515625" style="20" customWidth="1"/>
+    <col min="65" max="79" width="5.28515625" customWidth="1"/>
+    <col min="80" max="80" width="5.28515625" style="4" customWidth="1"/>
+    <col min="81" max="81" width="5.28515625" style="7" customWidth="1"/>
+    <col min="82" max="82" width="5.7109375" style="20" customWidth="1"/>
+    <col min="83" max="97" width="5.7109375" customWidth="1"/>
+    <col min="98" max="98" width="5.7109375" style="4" customWidth="1"/>
+    <col min="99" max="104" width="5.7109375" customWidth="1"/>
+    <col min="105" max="105" width="5.7109375" style="4" customWidth="1"/>
+    <col min="106" max="118" width="5.7109375" style="7" customWidth="1"/>
+    <col min="119" max="119" width="21.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="20.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="20.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="124" max="139" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:139">
@@ -9873,7 +9873,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:121" ht="28.8">
+    <row r="101" spans="1:121" ht="30">
       <c r="A101" t="s">
         <v>136</v>
       </c>
@@ -9935,7 +9935,7 @@
       <c r="DP101"/>
       <c r="DQ101"/>
     </row>
-    <row r="102" spans="1:121" ht="13.2" customHeight="1">
+    <row r="102" spans="1:121" ht="13.15" customHeight="1">
       <c r="A102" t="s">
         <v>136</v>
       </c>
@@ -9996,7 +9996,7 @@
       <c r="DP102"/>
       <c r="DQ102"/>
     </row>
-    <row r="103" spans="1:121" ht="13.2" customHeight="1">
+    <row r="103" spans="1:121" ht="13.15" customHeight="1">
       <c r="A103" t="s">
         <v>136</v>
       </c>
@@ -10051,7 +10051,7 @@
       <c r="DP103"/>
       <c r="DQ103"/>
     </row>
-    <row r="104" spans="1:121" ht="14.4" customHeight="1">
+    <row r="104" spans="1:121" ht="14.45" customHeight="1">
       <c r="A104" t="s">
         <v>136</v>
       </c>
@@ -10230,7 +10230,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:121" ht="13.95" customHeight="1">
+    <row r="107" spans="1:121" ht="13.9" customHeight="1">
       <c r="A107" t="s">
         <v>136</v>
       </c>
@@ -11873,7 +11873,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:123" ht="43.2">
+    <row r="133" spans="1:123" ht="60">
       <c r="A133" t="s">
         <v>217</v>
       </c>
@@ -11941,7 +11941,7 @@
       <c r="DP133"/>
       <c r="DQ133"/>
     </row>
-    <row r="134" spans="1:123" ht="43.2">
+    <row r="134" spans="1:123" ht="60">
       <c r="A134" t="s">
         <v>217</v>
       </c>
@@ -18324,12 +18324,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="1ff0e60b-5513-4fe6-897f-4cc6ed024994" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18507,18 +18506,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="1ff0e60b-5513-4fe6-897f-4cc6ed024994" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDA455DF-C4FA-4F8E-9198-EA78FE5B5EEF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BB0AF43-5131-40FC-A1A5-3DE82AC4E597}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
@@ -18541,7 +18539,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BB0AF43-5131-40FC-A1A5-3DE82AC4E597}">
-  <ds:schemaRefs/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDA455DF-C4FA-4F8E-9198-EA78FE5B5EEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>